<commit_message>
Store spreadsheet dates as midnight UTC
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/stock-messy.xlsx
+++ b/data/stock-messy.xlsx
@@ -1716,7 +1716,7 @@
         <v>21</v>
       </c>
       <c r="H3" s="1">
-        <v>46276.91666666667</v>
+        <v>46277</v>
       </c>
       <c r="J3" t="s">
         <v>22</v>
@@ -1768,7 +1768,7 @@
         <v>57.99</v>
       </c>
       <c r="H5" s="1">
-        <v>46189.91666666667</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1898,7 +1898,7 @@
         <v>50</v>
       </c>
       <c r="H10" s="1">
-        <v>46193.91666666667</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -1924,7 +1924,7 @@
         <v>54</v>
       </c>
       <c r="H11" s="1">
-        <v>46196.91666666667</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -2233,7 +2233,7 @@
         <v>108</v>
       </c>
       <c r="H23" s="1">
-        <v>46174.91666666667</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -2363,7 +2363,7 @@
         <v>126</v>
       </c>
       <c r="H28" s="1">
-        <v>46193.91666666667</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -2621,7 +2621,7 @@
         <v>108</v>
       </c>
       <c r="H38" s="1">
-        <v>46245.91666666667</v>
+        <v>46246</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
@@ -2751,7 +2751,7 @@
         <v>36.99</v>
       </c>
       <c r="H43" s="1">
-        <v>46134.91666666667</v>
+        <v>46135</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
@@ -2777,7 +2777,7 @@
         <v>198</v>
       </c>
       <c r="H44" s="1">
-        <v>46177.91666666667</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
@@ -2956,7 +2956,7 @@
         <v>163</v>
       </c>
       <c r="H51" s="1">
-        <v>46194.91666666667</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
@@ -3034,7 +3034,7 @@
         <v>242</v>
       </c>
       <c r="H54" s="1">
-        <v>46283.91666666667</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
@@ -3112,7 +3112,7 @@
         <v>254</v>
       </c>
       <c r="H57" s="1">
-        <v>46119.91666666667</v>
+        <v>46120</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
@@ -3369,7 +3369,7 @@
         <v>21</v>
       </c>
       <c r="H67" s="1">
-        <v>46151.91666666667</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
@@ -3395,7 +3395,7 @@
         <v>36.99</v>
       </c>
       <c r="H68" s="1">
-        <v>46134.91666666667</v>
+        <v>46135</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
@@ -3525,7 +3525,7 @@
         <v>318</v>
       </c>
       <c r="H73" s="1">
-        <v>46130.91666666667</v>
+        <v>46131</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
@@ -3551,7 +3551,7 @@
         <v>278</v>
       </c>
       <c r="H74" s="1">
-        <v>46237.91666666667</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
@@ -3577,7 +3577,7 @@
         <v>145</v>
       </c>
       <c r="H75" s="1">
-        <v>46176.91666666667</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
@@ -3629,7 +3629,7 @@
         <v>331</v>
       </c>
       <c r="H77" s="1">
-        <v>46136.91666666667</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
@@ -3941,7 +3941,7 @@
         <v>383</v>
       </c>
       <c r="H89" s="1">
-        <v>46281.91666666667</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.25">
@@ -3993,7 +3993,7 @@
         <v>21</v>
       </c>
       <c r="H91" s="1">
-        <v>46151.91666666667</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.25">
@@ -4019,7 +4019,7 @@
         <v>391</v>
       </c>
       <c r="H92" s="1">
-        <v>46275.91666666667</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Rename two invented suppliers that matched real companies
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/stock-messy.xlsx
+++ b/data/stock-messy.xlsx
@@ -70,7 +70,7 @@
     <t>KIT-0107</t>
   </si>
   <si>
-    <t>Kestrel Trading</t>
+    <t>Tidemill Wholesale</t>
   </si>
   <si>
     <t xml:space="preserve"> £ 15.00</t>
@@ -403,7 +403,7 @@
     <t>BED-0100</t>
   </si>
   <si>
-    <t>Northmere Textiles</t>
+    <t>Wrenfold Textiles</t>
   </si>
   <si>
     <t xml:space="preserve"> £ 10.00</t>
@@ -421,7 +421,7 @@
     <t>BED-0107</t>
   </si>
   <si>
-    <t>Northmere Textiles Ltd</t>
+    <t>Wrenfold Textiles Ltd</t>
   </si>
   <si>
     <t>8 May</t>

</xml_diff>